<commit_message>
added lists and triggers mostly
</commit_message>
<xml_diff>
--- a/ListsForDB/Department_Clean.xlsx
+++ b/ListsForDB/Department_Clean.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>dept_id</t>
   </si>
@@ -122,24 +122,6 @@
   </si>
   <si>
     <t>Περιγραφή τμήματος Ψυχιατρικό</t>
-  </si>
-  <si>
-    <t>A20000000005</t>
-  </si>
-  <si>
-    <t>A20000000014</t>
-  </si>
-  <si>
-    <t>A20000000016</t>
-  </si>
-  <si>
-    <t>A20000000022</t>
-  </si>
-  <si>
-    <t>A20000000026</t>
-  </si>
-  <si>
-    <t>A20000000029</t>
   </si>
 </sst>
 </file>
@@ -536,8 +518,8 @@
       <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
-        <v>36</v>
+      <c r="F2">
+        <v>20000000005</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -556,8 +538,8 @@
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3" t="s">
-        <v>37</v>
+      <c r="F3">
+        <v>20000000014</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -576,8 +558,8 @@
       <c r="E4">
         <v>2</v>
       </c>
-      <c r="F4" t="s">
-        <v>38</v>
+      <c r="F4">
+        <v>20000000016</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -596,8 +578,8 @@
       <c r="E5">
         <v>4</v>
       </c>
-      <c r="F5" t="s">
-        <v>39</v>
+      <c r="F5">
+        <v>20000000022</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -616,8 +598,8 @@
       <c r="E6">
         <v>2</v>
       </c>
-      <c r="F6" t="s">
-        <v>40</v>
+      <c r="F6">
+        <v>20000000026</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -636,8 +618,8 @@
       <c r="E7">
         <v>1</v>
       </c>
-      <c r="F7" t="s">
-        <v>41</v>
+      <c r="F7">
+        <v>20000000029</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -656,8 +638,8 @@
       <c r="E8">
         <v>4</v>
       </c>
-      <c r="F8" t="s">
-        <v>36</v>
+      <c r="F8">
+        <v>20000000005</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -676,8 +658,8 @@
       <c r="E9">
         <v>4</v>
       </c>
-      <c r="F9" t="s">
-        <v>37</v>
+      <c r="F9">
+        <v>20000000014</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -696,8 +678,8 @@
       <c r="E10">
         <v>1</v>
       </c>
-      <c r="F10" t="s">
-        <v>38</v>
+      <c r="F10">
+        <v>20000000016</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -716,8 +698,8 @@
       <c r="E11">
         <v>4</v>
       </c>
-      <c r="F11" t="s">
-        <v>39</v>
+      <c r="F11">
+        <v>20000000022</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -736,8 +718,8 @@
       <c r="E12">
         <v>0</v>
       </c>
-      <c r="F12" t="s">
-        <v>40</v>
+      <c r="F12">
+        <v>20000000026</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -756,8 +738,8 @@
       <c r="E13">
         <v>0</v>
       </c>
-      <c r="F13" t="s">
-        <v>41</v>
+      <c r="F13">
+        <v>20000000029</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -776,8 +758,8 @@
       <c r="E14">
         <v>4</v>
       </c>
-      <c r="F14" t="s">
-        <v>36</v>
+      <c r="F14">
+        <v>20000000005</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -796,8 +778,8 @@
       <c r="E15">
         <v>0</v>
       </c>
-      <c r="F15" t="s">
-        <v>37</v>
+      <c r="F15">
+        <v>20000000014</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -816,8 +798,8 @@
       <c r="E16">
         <v>1</v>
       </c>
-      <c r="F16" t="s">
-        <v>38</v>
+      <c r="F16">
+        <v>20000000016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>